<commit_message>
Add verified Iraqi telecom personnel source
</commit_message>
<xml_diff>
--- a/政府人员监控矩阵_v1.0.xlsx
+++ b/政府人员监控矩阵_v1.0.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R74ddd4c9407e4b36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="伊拉克" sheetId="2" r:id="Rf080f7da49ca47af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="约旦" sheetId="3" r:id="R65ddd1a7f4f8492f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黎巴嫩" sheetId="4" r:id="Rfe91447f669e4e85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R769b947242324530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="伊拉克" sheetId="2" r:id="Rf9af9032132a4d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="约旦" sheetId="3" r:id="Rea8e0214be6a4675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黎巴嫩" sheetId="4" r:id="R0782ccf637184353"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -850,13 +850,13 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="C4" s="42" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D4" s="42" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E4" s="42" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F4" s="42" t="str">
         <x:v>https://www.cabinet.iq/</x:v>
@@ -1244,17 +1244,19 @@
         <x:v>伊拉克</x:v>
       </x:c>
       <x:c r="C9" s="74" t="str">
-        <x:v>待官方核验</x:v>
+        <x:v>Mustafa Sanad</x:v>
       </x:c>
       <x:c r="D9" s="74" t="str">
         <x:v>通信部长</x:v>
       </x:c>
-      <x:c r="E9" s="74" t="str"/>
+      <x:c r="E9" s="74" t="str">
+        <x:v>https://t.me/mociraq2023</x:v>
+      </x:c>
       <x:c r="F9" s="74" t="str"/>
       <x:c r="G9" s="74" t="str"/>
       <x:c r="H9" s="74" t="str"/>
       <x:c r="I9" s="73" t="str">
-        <x:v>待核验</x:v>
+        <x:v>机构账号已核验</x:v>
       </x:c>
       <x:c r="J9" s="73" t="str">
         <x:v>在任</x:v>
@@ -1874,7 +1876,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3668bb6b304b44ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb21c289d9eff41c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2977,7 +2979,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2066949b3f3d483f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa46f3f478134a42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3882,7 +3884,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf0a2626e77f402f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc29403f031a44079"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>